<commit_message>
Complete Accounts QA testing and traceability
</commit_message>
<xml_diff>
--- a/03-Test-Cases/Detailed-test-cases/EspoCRM-Login-Test-Cases-v1.0.xlsx
+++ b/03-Test-Cases/Detailed-test-cases/EspoCRM-Login-Test-Cases-v1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDIQ\EspoCRM-QA-Automation\03-Test-Cases\Detailed-test-cases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE5BBD8-4284-45CC-882B-EB5B2A147A42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B06A7F-02CB-418A-BEBA-0AE433127CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="80">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -299,6 +299,24 @@
   </si>
   <si>
     <t>Password: Valid test password</t>
+  </si>
+  <si>
+    <t>Actual Result</t>
+  </si>
+  <si>
+    <t>Login page loaded successfully aand displayed the username and password fields and login control.</t>
+  </si>
+  <si>
+    <t>User successfully authenticated and redirected to EspoCRM application</t>
+  </si>
+  <si>
+    <t>Application successfully rejected the login attempt and displayed an appropriate authentication/validation message.</t>
+  </si>
+  <si>
+    <t>Password charcaters successfully masked and didn't displpayed as pplain text.</t>
+  </si>
+  <si>
+    <t>User successfully logged out and no longer have access to authenticated pages without logging in again.</t>
   </si>
 </sst>
 </file>
@@ -339,12 +357,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -625,7 +642,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
@@ -638,10 +655,11 @@
     <col min="8" max="8" width="8.44140625" customWidth="1"/>
     <col min="9" max="9" width="7.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="26.77734375" customWidth="1"/>
+    <col min="12" max="12" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -673,10 +691,13 @@
         <v>9</v>
       </c>
       <c r="K1" t="s">
+        <v>74</v>
+      </c>
+      <c r="L1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="49.8" customHeight="1">
+    <row r="2" spans="1:12" ht="57.6">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -698,20 +719,23 @@
       <c r="G2" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="J2" s="2" t="s">
+      <c r="H2" t="s">
+        <v>37</v>
+      </c>
+      <c r="I2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" t="s">
         <v>38</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="L2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="72">
+    <row r="3" spans="1:12" ht="72">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -743,10 +767,13 @@
         <v>67</v>
       </c>
       <c r="K3" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="57.6">
+    <row r="4" spans="1:12" ht="72">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -777,11 +804,14 @@
       <c r="J4" t="s">
         <v>45</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="57.6">
+    <row r="5" spans="1:12" ht="72">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -812,11 +842,14 @@
       <c r="J5" t="s">
         <v>45</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="57.6">
+    <row r="6" spans="1:12" ht="72">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -847,11 +880,14 @@
       <c r="J6" t="s">
         <v>45</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="72">
+    <row r="7" spans="1:12" ht="72">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -882,11 +918,14 @@
       <c r="J7" t="s">
         <v>45</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="72">
+    <row r="8" spans="1:12" ht="72">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -917,11 +956,14 @@
       <c r="J8" t="s">
         <v>45</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L8" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="86.4">
+    <row r="9" spans="1:12" ht="86.4">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -952,11 +994,14 @@
       <c r="J9" t="s">
         <v>45</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="86.4">
+    <row r="10" spans="1:12" ht="86.4">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -978,7 +1023,7 @@
       <c r="G10" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" t="s">
         <v>59</v>
       </c>
       <c r="I10" s="1" t="s">
@@ -987,11 +1032,14 @@
       <c r="J10" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="L10" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="72">
+    <row r="11" spans="1:12" ht="72">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -1022,7 +1070,10 @@
       <c r="J11" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="L11" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>